<commit_message>
Update Excel financial model template
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bizplan-ecommerce/skills/ecommerce-financial-model/templates/eCommerce Model v1.xlsx
+++ b/bizplan-ecommerce/skills/ecommerce-financial-model/templates/eCommerce Model v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adurex/Documents/bizplan-plugin/bizplan-ecommerce/skills/ecommerce-financial-model/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16A451B-EF47-4A47-98FB-BA1A838BD694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EC3D578-B3CA-C645-8F84-66CACC86447C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16540" tabRatio="634" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16540" tabRatio="634" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumptions" sheetId="5" r:id="rId1"/>
@@ -8932,7 +8932,7 @@
       <c r="B107" s="32"/>
       <c r="D107" s="87"/>
       <c r="E107" s="25">
-        <f>$D$104/D103</f>
+        <f>IF(D103=0,0,$D$104/D103)</f>
         <v>3.0416666666666665</v>
       </c>
       <c r="F107" s="25">
@@ -10541,27 +10541,27 @@
         <v>18</v>
       </c>
       <c r="E177" s="3">
-        <f t="shared" ref="E177:J177" si="45">E142/E107</f>
+        <f>IF(E107=0,0,E142/E107)</f>
         <v>310787.67123287672</v>
       </c>
       <c r="F177" s="3">
-        <f t="shared" si="45"/>
+        <f>IF(F107=0,0,F142/F107)</f>
         <v>530747.64554794517</v>
       </c>
       <c r="G177" s="3">
-        <f t="shared" si="45"/>
+        <f>IF(G107=0,0,G142/G107)</f>
         <v>808035.5991652396</v>
       </c>
       <c r="H177" s="3">
-        <f t="shared" si="45"/>
+        <f>IF(H107=0,0,H142/H107)</f>
         <v>1156434.0262193638</v>
       </c>
       <c r="I177" s="3">
-        <f t="shared" si="45"/>
+        <f>IF(I107=0,0,I142/I107)</f>
         <v>1593022.4992052065</v>
       </c>
       <c r="J177" s="3">
-        <f t="shared" si="45"/>
+        <f>IF(J107=0,0,J142/J107)</f>
         <v>2138970.698209051</v>
       </c>
       <c r="K177"/>
@@ -10581,23 +10581,23 @@
         <v>418207.8339041096</v>
       </c>
       <c r="F178" s="15">
-        <f t="shared" ref="F178:J178" si="46">SUM(F175:F177)</f>
+        <f t="shared" ref="F178:J178" si="45">SUM(F175:F177)</f>
         <v>209718.84267979453</v>
       </c>
       <c r="G178" s="15">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>215464.3996507586</v>
       </c>
       <c r="H178" s="15">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>560714.09572101396</v>
       </c>
       <c r="I178" s="15">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>1445336.653835102</v>
       </c>
       <c r="J178" s="15">
-        <f t="shared" si="46"/>
+        <f t="shared" si="45"/>
         <v>3189379.3297813004</v>
       </c>
       <c r="K178"/>
@@ -10614,23 +10614,23 @@
         <v>151250</v>
       </c>
       <c r="F179" s="3">
-        <f t="shared" ref="F179:J179" si="47">F241</f>
+        <f t="shared" ref="F179:J179" si="46">F241</f>
         <v>400434.375</v>
       </c>
       <c r="G179" s="3">
-        <f t="shared" si="47"/>
+        <f t="shared" si="46"/>
         <v>776359.06562500005</v>
       </c>
       <c r="H179" s="3">
-        <f t="shared" si="47"/>
+        <f t="shared" si="46"/>
         <v>1317439.3148468751</v>
       </c>
       <c r="I179" s="3">
-        <f t="shared" si="47"/>
+        <f t="shared" si="46"/>
         <v>2075137.9458064411</v>
       </c>
       <c r="J179" s="3">
-        <f t="shared" si="47"/>
+        <f t="shared" si="46"/>
         <v>3011177.1978085707</v>
       </c>
       <c r="K179"/>
@@ -10646,27 +10646,27 @@
       <c r="C180" s="27"/>
       <c r="D180" s="27"/>
       <c r="E180" s="27">
-        <f t="shared" ref="E180:J180" si="48">SUM(E178:E179)</f>
+        <f t="shared" ref="E180:J180" si="47">SUM(E178:E179)</f>
         <v>569457.83390410966</v>
       </c>
       <c r="F180" s="27">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>610153.21767979453</v>
       </c>
       <c r="G180" s="27">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>991823.46527575864</v>
       </c>
       <c r="H180" s="27">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>1878153.410567889</v>
       </c>
       <c r="I180" s="27">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>3520474.5996415429</v>
       </c>
       <c r="J180" s="27">
-        <f t="shared" si="48"/>
+        <f t="shared" si="47"/>
         <v>6200556.5275898706</v>
       </c>
       <c r="K180"/>
@@ -10706,27 +10706,27 @@
         <v>128</v>
       </c>
       <c r="E184" s="3">
-        <f t="shared" ref="E184:J184" si="49">(E151+E142)*$D$110/$D$104</f>
+        <f t="shared" ref="E184:J184" si="48">(E151+E142)*$D$110/$D$104</f>
         <v>96035.95890410959</v>
       </c>
       <c r="F184" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="48"/>
         <v>175207.99892979453</v>
       </c>
       <c r="G184" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="48"/>
         <v>287919.70343601238</v>
       </c>
       <c r="H184" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="48"/>
         <v>446774.30740984518</v>
       </c>
       <c r="I184" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="48"/>
         <v>668958.49876932276</v>
       </c>
       <c r="J184" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="48"/>
         <v>977897.08195268747</v>
       </c>
       <c r="K184"/>
@@ -10742,27 +10742,27 @@
       <c r="C185" s="15"/>
       <c r="D185" s="15"/>
       <c r="E185" s="15">
-        <f t="shared" ref="E185:J185" si="50">SUM(E184:E184)</f>
+        <f t="shared" ref="E185:J185" si="49">SUM(E184:E184)</f>
         <v>96035.95890410959</v>
       </c>
       <c r="F185" s="15">
-        <f t="shared" si="50"/>
+        <f t="shared" si="49"/>
         <v>175207.99892979453</v>
       </c>
       <c r="G185" s="15">
-        <f t="shared" si="50"/>
+        <f t="shared" si="49"/>
         <v>287919.70343601238</v>
       </c>
       <c r="H185" s="15">
-        <f t="shared" si="50"/>
+        <f t="shared" si="49"/>
         <v>446774.30740984518</v>
       </c>
       <c r="I185" s="15">
-        <f t="shared" si="50"/>
+        <f t="shared" si="49"/>
         <v>668958.49876932276</v>
       </c>
       <c r="J185" s="15">
-        <f t="shared" si="50"/>
+        <f t="shared" si="49"/>
         <v>977897.08195268747</v>
       </c>
       <c r="K185"/>
@@ -10779,23 +10779,23 @@
         <v>0</v>
       </c>
       <c r="F186" s="3">
-        <f t="shared" ref="F186:J186" si="51">F251</f>
+        <f t="shared" ref="F186:J186" si="50">F251</f>
         <v>0</v>
       </c>
       <c r="G186" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="50"/>
         <v>0</v>
       </c>
       <c r="H186" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="50"/>
         <v>0</v>
       </c>
       <c r="I186" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="50"/>
         <v>0</v>
       </c>
       <c r="J186" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="50"/>
         <v>0</v>
       </c>
       <c r="K186"/>
@@ -10815,23 +10815,23 @@
         <v>96035.95890410959</v>
       </c>
       <c r="F187" s="15">
-        <f t="shared" ref="F187:J187" si="52">SUM(F185:F186)</f>
+        <f t="shared" ref="F187:J187" si="51">SUM(F185:F186)</f>
         <v>175207.99892979453</v>
       </c>
       <c r="G187" s="15">
-        <f t="shared" si="52"/>
+        <f t="shared" si="51"/>
         <v>287919.70343601238</v>
       </c>
       <c r="H187" s="15">
-        <f t="shared" si="52"/>
+        <f t="shared" si="51"/>
         <v>446774.30740984518</v>
       </c>
       <c r="I187" s="15">
-        <f t="shared" si="52"/>
+        <f t="shared" si="51"/>
         <v>668958.49876932276</v>
       </c>
       <c r="J187" s="15">
-        <f t="shared" si="52"/>
+        <f t="shared" si="51"/>
         <v>977897.08195268747</v>
       </c>
       <c r="K187"/>
@@ -10861,19 +10861,19 @@
         <v>500000</v>
       </c>
       <c r="G189" s="3">
-        <f t="shared" ref="G189:J189" si="53">+F189</f>
+        <f t="shared" ref="G189:J189" si="52">+F189</f>
         <v>500000</v>
       </c>
       <c r="H189" s="3">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>500000</v>
       </c>
       <c r="I189" s="3">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>500000</v>
       </c>
       <c r="J189" s="3">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>500000</v>
       </c>
       <c r="K189"/>
@@ -10886,27 +10886,27 @@
         <v>131</v>
       </c>
       <c r="E190" s="3">
-        <f t="shared" ref="E190:J190" si="54">+D190+E167-E169</f>
+        <f t="shared" ref="E190:J190" si="53">+D190+E167-E169</f>
         <v>-26578.125</v>
       </c>
       <c r="F190" s="3">
-        <f t="shared" si="54"/>
+        <f t="shared" si="53"/>
         <v>-65054.78125</v>
       </c>
       <c r="G190" s="3">
-        <f t="shared" si="54"/>
+        <f t="shared" si="53"/>
         <v>203903.76183974621</v>
       </c>
       <c r="H190" s="3">
-        <f t="shared" si="54"/>
+        <f t="shared" si="53"/>
         <v>931379.1031580437</v>
       </c>
       <c r="I190" s="3">
-        <f t="shared" si="54"/>
+        <f t="shared" si="53"/>
         <v>2351516.1008722205</v>
       </c>
       <c r="J190" s="3">
-        <f t="shared" si="54"/>
+        <f t="shared" si="53"/>
         <v>4722659.4456371833</v>
       </c>
       <c r="K190"/>
@@ -10926,23 +10926,23 @@
         <v>473421.875</v>
       </c>
       <c r="F191" s="15">
-        <f t="shared" ref="F191:J191" si="55">SUM(F189:F190)</f>
+        <f t="shared" ref="F191:J191" si="54">SUM(F189:F190)</f>
         <v>434945.21875</v>
       </c>
       <c r="G191" s="15">
-        <f t="shared" si="55"/>
+        <f t="shared" si="54"/>
         <v>703903.76183974626</v>
       </c>
       <c r="H191" s="15">
-        <f t="shared" si="55"/>
+        <f t="shared" si="54"/>
         <v>1431379.1031580437</v>
       </c>
       <c r="I191" s="15">
-        <f t="shared" si="55"/>
+        <f t="shared" si="54"/>
         <v>2851516.1008722205</v>
       </c>
       <c r="J191" s="15">
-        <f t="shared" si="55"/>
+        <f t="shared" si="54"/>
         <v>5222659.4456371833</v>
       </c>
       <c r="K191"/>
@@ -10962,23 +10962,23 @@
         <v>569457.83390410955</v>
       </c>
       <c r="F192" s="27">
-        <f t="shared" ref="F192:J192" si="56">+F191+F187</f>
+        <f t="shared" ref="F192:J192" si="55">+F191+F187</f>
         <v>610153.21767979453</v>
       </c>
       <c r="G192" s="27">
-        <f t="shared" si="56"/>
+        <f t="shared" si="55"/>
         <v>991823.46527575864</v>
       </c>
       <c r="H192" s="27">
-        <f t="shared" si="56"/>
+        <f t="shared" si="55"/>
         <v>1878153.410567889</v>
       </c>
       <c r="I192" s="27">
-        <f t="shared" si="56"/>
+        <f t="shared" si="55"/>
         <v>3520474.5996415433</v>
       </c>
       <c r="J192" s="27">
-        <f t="shared" si="56"/>
+        <f t="shared" si="55"/>
         <v>6200556.5275898706</v>
       </c>
       <c r="K192"/>
@@ -11005,27 +11005,27 @@
         <v>132</v>
       </c>
       <c r="E194" s="29">
-        <f t="shared" ref="E194:J194" si="57">E192-E180</f>
+        <f t="shared" ref="E194:J194" si="56">E192-E180</f>
         <v>0</v>
       </c>
       <c r="F194" s="29">
-        <f t="shared" si="57"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="G194" s="29">
-        <f t="shared" si="57"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="H194" s="29">
-        <f t="shared" si="57"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="I194" s="29">
-        <f t="shared" si="57"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="J194" s="29">
-        <f t="shared" si="57"/>
+        <f t="shared" si="56"/>
         <v>0</v>
       </c>
       <c r="K194"/>
@@ -11084,27 +11084,27 @@
         <v>120</v>
       </c>
       <c r="E199" s="3">
-        <f t="shared" ref="E199:J199" si="58">E167</f>
+        <f t="shared" ref="E199:J199" si="57">E167</f>
         <v>-26578.125</v>
       </c>
       <c r="F199" s="3">
-        <f t="shared" si="58"/>
+        <f t="shared" si="57"/>
         <v>-38476.65625</v>
       </c>
       <c r="G199" s="3">
-        <f t="shared" si="58"/>
+        <f t="shared" si="57"/>
         <v>268958.54308974621</v>
       </c>
       <c r="H199" s="3">
-        <f t="shared" si="58"/>
+        <f t="shared" si="57"/>
         <v>727475.34131829755</v>
       </c>
       <c r="I199" s="3">
-        <f t="shared" si="58"/>
+        <f t="shared" si="57"/>
         <v>1420136.9977141765</v>
       </c>
       <c r="J199" s="3">
-        <f t="shared" si="58"/>
+        <f t="shared" si="57"/>
         <v>2371143.3447649633</v>
       </c>
       <c r="K199"/>
@@ -11117,27 +11117,27 @@
         <v>7</v>
       </c>
       <c r="E200" s="3">
-        <f t="shared" ref="E200:J200" si="59">E162</f>
+        <f t="shared" ref="E200:J200" si="58">E162</f>
         <v>37812.5</v>
       </c>
       <c r="F200" s="3">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>109561.71875</v>
       </c>
       <c r="G200" s="3">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>230933.32109375001</v>
       </c>
       <c r="H200" s="3">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>423936.71367265622</v>
       </c>
       <c r="I200" s="3">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>719345.54983071168</v>
       </c>
       <c r="J200" s="3">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>1267566.5241225134</v>
       </c>
       <c r="K200"/>
@@ -11159,27 +11159,27 @@
         <v>124</v>
       </c>
       <c r="E202" s="3">
-        <f t="shared" ref="E202:J203" si="60">E176-D176</f>
+        <f t="shared" ref="E202:J203" si="59">E176-D176</f>
         <v>19968.107876712329</v>
       </c>
       <c r="F202" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>17921.376819349312</v>
       </c>
       <c r="G202" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>26204.697089576206</v>
       </c>
       <c r="H202" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>37827.472788565385</v>
       </c>
       <c r="I202" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>54078.491095564459</v>
       </c>
       <c r="J202" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>76736.847945588437</v>
       </c>
       <c r="K202"/>
@@ -11192,27 +11192,27 @@
         <v>18</v>
       </c>
       <c r="E203" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>310787.67123287672</v>
       </c>
       <c r="F203" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>219959.97431506845</v>
       </c>
       <c r="G203" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>277287.95361729444</v>
       </c>
       <c r="H203" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>348398.42705412419</v>
       </c>
       <c r="I203" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>436588.47298584273</v>
       </c>
       <c r="J203" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="59"/>
         <v>545948.19900384452</v>
       </c>
       <c r="K203"/>
@@ -11229,23 +11229,23 @@
         <v>96035.95890410959</v>
       </c>
       <c r="F204" s="3">
-        <f t="shared" ref="F204:J204" si="61">F184-E184</f>
+        <f t="shared" ref="F204:J204" si="60">F184-E184</f>
         <v>79172.040025684939</v>
       </c>
       <c r="G204" s="3">
-        <f t="shared" si="61"/>
+        <f t="shared" si="60"/>
         <v>112711.70450621785</v>
       </c>
       <c r="H204" s="3">
-        <f t="shared" si="61"/>
+        <f t="shared" si="60"/>
         <v>158854.6039738328</v>
       </c>
       <c r="I204" s="3">
-        <f t="shared" si="61"/>
+        <f t="shared" si="60"/>
         <v>222184.19135947758</v>
       </c>
       <c r="J204" s="3">
-        <f t="shared" si="61"/>
+        <f t="shared" si="60"/>
         <v>308938.58318336471</v>
       </c>
       <c r="K204"/>
@@ -11265,23 +11265,23 @@
         <v>-223485.44520547945</v>
       </c>
       <c r="F205" s="15">
-        <f t="shared" ref="F205:J205" si="62">F199+F200-F202-F203+F204</f>
+        <f t="shared" ref="F205:J205" si="61">F199+F200-F202-F203+F204</f>
         <v>-87624.248608732814</v>
       </c>
       <c r="G205" s="15">
-        <f t="shared" si="62"/>
+        <f t="shared" si="61"/>
         <v>309110.91798284341</v>
       </c>
       <c r="H205" s="15">
-        <f t="shared" si="62"/>
+        <f t="shared" si="61"/>
         <v>924040.75912209705</v>
       </c>
       <c r="I205" s="15">
-        <f t="shared" si="62"/>
+        <f t="shared" si="61"/>
         <v>1870999.7748229585</v>
       </c>
       <c r="J205" s="15">
-        <f t="shared" si="62"/>
+        <f t="shared" si="61"/>
         <v>3324963.4051214084</v>
       </c>
       <c r="K205"/>
@@ -11309,27 +11309,27 @@
         <v>141</v>
       </c>
       <c r="E208" s="3">
-        <f t="shared" ref="E208:J208" si="63">E116</f>
+        <f t="shared" ref="E208:J208" si="62">E116</f>
         <v>189062.5</v>
       </c>
       <c r="F208" s="3">
-        <f t="shared" si="63"/>
+        <f t="shared" si="62"/>
         <v>358746.09375</v>
       </c>
       <c r="G208" s="3">
-        <f t="shared" si="63"/>
+        <f t="shared" si="62"/>
         <v>606858.01171875</v>
       </c>
       <c r="H208" s="3">
-        <f t="shared" si="63"/>
+        <f t="shared" si="62"/>
         <v>965016.9628945312</v>
       </c>
       <c r="I208" s="3">
-        <f t="shared" si="63"/>
+        <f t="shared" si="62"/>
         <v>1477044.1807902777</v>
       </c>
       <c r="J208" s="3">
-        <f t="shared" si="63"/>
+        <f t="shared" si="62"/>
         <v>2203605.7761246427</v>
       </c>
       <c r="K208"/>
@@ -11345,27 +11345,27 @@
       <c r="C209" s="15"/>
       <c r="D209" s="15"/>
       <c r="E209" s="15">
-        <f t="shared" ref="E209:J209" si="64">SUM(E208:E208)</f>
+        <f t="shared" ref="E209:J209" si="63">SUM(E208:E208)</f>
         <v>189062.5</v>
       </c>
       <c r="F209" s="15">
-        <f t="shared" si="64"/>
+        <f t="shared" si="63"/>
         <v>358746.09375</v>
       </c>
       <c r="G209" s="15">
-        <f t="shared" si="64"/>
+        <f t="shared" si="63"/>
         <v>606858.01171875</v>
       </c>
       <c r="H209" s="15">
-        <f t="shared" si="64"/>
+        <f t="shared" si="63"/>
         <v>965016.9628945312</v>
       </c>
       <c r="I209" s="15">
-        <f t="shared" si="64"/>
+        <f t="shared" si="63"/>
         <v>1477044.1807902777</v>
       </c>
       <c r="J209" s="15">
-        <f t="shared" si="64"/>
+        <f t="shared" si="63"/>
         <v>2203605.7761246427</v>
       </c>
       <c r="K209"/>
@@ -11410,23 +11410,23 @@
         <v>0</v>
       </c>
       <c r="F213" s="3">
-        <f t="shared" ref="F213:J213" si="65">F250</f>
+        <f t="shared" ref="F213:J213" si="64">F250</f>
         <v>0</v>
       </c>
       <c r="G213" s="3">
-        <f t="shared" si="65"/>
+        <f t="shared" si="64"/>
         <v>0</v>
       </c>
       <c r="H213" s="3">
-        <f t="shared" si="65"/>
+        <f t="shared" si="64"/>
         <v>0</v>
       </c>
       <c r="I213" s="3">
-        <f t="shared" si="65"/>
+        <f t="shared" si="64"/>
         <v>0</v>
       </c>
       <c r="J213" s="3">
-        <f t="shared" si="65"/>
+        <f t="shared" si="64"/>
         <v>0</v>
       </c>
       <c r="K213"/>
@@ -11443,23 +11443,23 @@
         <v>0</v>
       </c>
       <c r="F214" s="3">
-        <f t="shared" ref="F214:J214" si="66">F212+F213</f>
+        <f t="shared" ref="F214:J214" si="65">F212+F213</f>
         <v>0</v>
       </c>
       <c r="G214" s="3">
-        <f t="shared" si="66"/>
+        <f t="shared" si="65"/>
         <v>0</v>
       </c>
       <c r="H214" s="3">
-        <f t="shared" si="66"/>
+        <f t="shared" si="65"/>
         <v>0</v>
       </c>
       <c r="I214" s="3">
-        <f t="shared" si="66"/>
+        <f t="shared" si="65"/>
         <v>0</v>
       </c>
       <c r="J214" s="3">
-        <f t="shared" si="66"/>
+        <f t="shared" si="65"/>
         <v>0</v>
       </c>
       <c r="K214"/>
@@ -11480,19 +11480,19 @@
         <v>0</v>
       </c>
       <c r="G215" s="3">
-        <f t="shared" ref="G215:J215" si="67">G189-F189</f>
+        <f t="shared" ref="G215:J215" si="66">G189-F189</f>
         <v>0</v>
       </c>
       <c r="H215" s="3">
-        <f t="shared" si="67"/>
+        <f t="shared" si="66"/>
         <v>0</v>
       </c>
       <c r="I215" s="3">
-        <f t="shared" si="67"/>
+        <f t="shared" si="66"/>
         <v>0</v>
       </c>
       <c r="J215" s="3">
-        <f t="shared" si="67"/>
+        <f t="shared" si="66"/>
         <v>0</v>
       </c>
       <c r="K215"/>
@@ -11505,27 +11505,27 @@
         <v>49</v>
       </c>
       <c r="E216" s="3">
-        <f t="shared" ref="E216:J216" si="68">E169</f>
+        <f t="shared" ref="E216:J216" si="67">E169</f>
         <v>0</v>
       </c>
       <c r="F216" s="3">
-        <f t="shared" si="68"/>
+        <f t="shared" si="67"/>
         <v>0</v>
       </c>
       <c r="G216" s="3">
-        <f t="shared" si="68"/>
+        <f t="shared" si="67"/>
         <v>0</v>
       </c>
       <c r="H216" s="3">
-        <f t="shared" si="68"/>
+        <f t="shared" si="67"/>
         <v>0</v>
       </c>
       <c r="I216" s="3">
-        <f t="shared" si="68"/>
+        <f t="shared" si="67"/>
         <v>0</v>
       </c>
       <c r="J216" s="3">
-        <f t="shared" si="68"/>
+        <f t="shared" si="67"/>
         <v>0</v>
       </c>
       <c r="K216"/>
@@ -11542,23 +11542,23 @@
         <v>500000</v>
       </c>
       <c r="F217" s="3">
-        <f t="shared" ref="F217:J217" si="69">F215-F216</f>
+        <f t="shared" ref="F217:J217" si="68">F215-F216</f>
         <v>0</v>
       </c>
       <c r="G217" s="3">
-        <f t="shared" si="69"/>
+        <f t="shared" si="68"/>
         <v>0</v>
       </c>
       <c r="H217" s="3">
-        <f t="shared" si="69"/>
+        <f t="shared" si="68"/>
         <v>0</v>
       </c>
       <c r="I217" s="3">
-        <f t="shared" si="69"/>
+        <f t="shared" si="68"/>
         <v>0</v>
       </c>
       <c r="J217" s="3">
-        <f t="shared" si="69"/>
+        <f t="shared" si="68"/>
         <v>0</v>
       </c>
       <c r="K217"/>
@@ -11578,23 +11578,23 @@
         <v>500000</v>
       </c>
       <c r="F218" s="15">
-        <f t="shared" ref="F218:J218" si="70">F217+F214</f>
+        <f t="shared" ref="F218:J218" si="69">F217+F214</f>
         <v>0</v>
       </c>
       <c r="G218" s="15">
-        <f t="shared" si="70"/>
+        <f t="shared" si="69"/>
         <v>0</v>
       </c>
       <c r="H218" s="15">
-        <f t="shared" si="70"/>
+        <f t="shared" si="69"/>
         <v>0</v>
       </c>
       <c r="I218" s="15">
-        <f t="shared" si="70"/>
+        <f t="shared" si="69"/>
         <v>0</v>
       </c>
       <c r="J218" s="15">
-        <f t="shared" si="70"/>
+        <f t="shared" si="69"/>
         <v>0</v>
       </c>
       <c r="K218"/>
@@ -11619,23 +11619,23 @@
         <v>0</v>
       </c>
       <c r="F220" s="17">
-        <f t="shared" ref="F220:J220" si="71">E222</f>
+        <f t="shared" ref="F220:J220" si="70">E222</f>
         <v>87452.054794520547</v>
       </c>
       <c r="G220" s="17">
-        <f t="shared" si="71"/>
+        <f t="shared" si="70"/>
         <v>-358918.28756421228</v>
       </c>
       <c r="H220" s="17">
-        <f t="shared" si="71"/>
+        <f t="shared" si="70"/>
         <v>-656665.38130011887</v>
       </c>
       <c r="I220" s="17">
-        <f t="shared" si="71"/>
+        <f t="shared" si="70"/>
         <v>-697641.58507255302</v>
       </c>
       <c r="J220" s="17">
-        <f t="shared" si="71"/>
+        <f t="shared" si="70"/>
         <v>-303685.99103987217</v>
       </c>
       <c r="K220"/>
@@ -11648,27 +11648,27 @@
         <v>136</v>
       </c>
       <c r="E221" s="3">
-        <f t="shared" ref="E221:J221" si="72">E205-E209+E218</f>
+        <f t="shared" ref="E221:J221" si="71">E205-E209+E218</f>
         <v>87452.054794520547</v>
       </c>
       <c r="F221" s="3">
-        <f t="shared" si="72"/>
+        <f t="shared" si="71"/>
         <v>-446370.34235873283</v>
       </c>
       <c r="G221" s="3">
-        <f t="shared" si="72"/>
+        <f t="shared" si="71"/>
         <v>-297747.09373590659</v>
       </c>
       <c r="H221" s="3">
-        <f t="shared" si="72"/>
+        <f t="shared" si="71"/>
         <v>-40976.20377243415</v>
       </c>
       <c r="I221" s="3">
-        <f t="shared" si="72"/>
+        <f t="shared" si="71"/>
         <v>393955.59403268085</v>
       </c>
       <c r="J221" s="3">
-        <f t="shared" si="72"/>
+        <f t="shared" si="71"/>
         <v>1121357.6289967657</v>
       </c>
       <c r="K221"/>
@@ -11688,23 +11688,23 @@
         <v>87452.054794520547</v>
       </c>
       <c r="F222" s="17">
-        <f t="shared" ref="F222:J222" si="73">SUM(F220:F221)</f>
+        <f t="shared" ref="F222:J222" si="72">SUM(F220:F221)</f>
         <v>-358918.28756421228</v>
       </c>
       <c r="G222" s="17">
-        <f t="shared" si="73"/>
+        <f t="shared" si="72"/>
         <v>-656665.38130011887</v>
       </c>
       <c r="H222" s="17">
-        <f t="shared" si="73"/>
+        <f t="shared" si="72"/>
         <v>-697641.58507255302</v>
       </c>
       <c r="I222" s="17">
-        <f t="shared" si="73"/>
+        <f t="shared" si="72"/>
         <v>-303685.99103987217</v>
       </c>
       <c r="J222" s="17">
-        <f t="shared" si="73"/>
+        <f t="shared" si="72"/>
         <v>817671.63795689354</v>
       </c>
       <c r="K222"/>
@@ -11766,27 +11766,27 @@
       </c>
       <c r="B227" s="30"/>
       <c r="E227" s="3">
-        <f t="shared" ref="E227:J227" si="74">D241</f>
+        <f t="shared" ref="E227:J227" si="73">D241</f>
         <v>0</v>
       </c>
       <c r="F227" s="3">
-        <f t="shared" si="74"/>
+        <f t="shared" si="73"/>
         <v>151250</v>
       </c>
       <c r="G227" s="3">
-        <f t="shared" si="74"/>
+        <f t="shared" si="73"/>
         <v>400434.375</v>
       </c>
       <c r="H227" s="3">
-        <f t="shared" si="74"/>
+        <f t="shared" si="73"/>
         <v>776359.06562500005</v>
       </c>
       <c r="I227" s="3">
-        <f t="shared" si="74"/>
+        <f t="shared" si="73"/>
         <v>1317439.3148468751</v>
       </c>
       <c r="J227" s="3">
-        <f t="shared" si="74"/>
+        <f t="shared" si="73"/>
         <v>2075137.9458064411</v>
       </c>
       <c r="K227"/>
@@ -11800,27 +11800,27 @@
       </c>
       <c r="B228" s="31"/>
       <c r="E228" s="3">
-        <f t="shared" ref="E228:J228" si="75">E116</f>
+        <f t="shared" ref="E228:J228" si="74">E116</f>
         <v>189062.5</v>
       </c>
       <c r="F228" s="3">
-        <f t="shared" si="75"/>
+        <f t="shared" si="74"/>
         <v>358746.09375</v>
       </c>
       <c r="G228" s="3">
-        <f t="shared" si="75"/>
+        <f t="shared" si="74"/>
         <v>606858.01171875</v>
       </c>
       <c r="H228" s="3">
-        <f t="shared" si="75"/>
+        <f t="shared" si="74"/>
         <v>965016.9628945312</v>
       </c>
       <c r="I228" s="3">
-        <f t="shared" si="75"/>
+        <f t="shared" si="74"/>
         <v>1477044.1807902777</v>
       </c>
       <c r="J228" s="3">
-        <f t="shared" si="75"/>
+        <f t="shared" si="74"/>
         <v>2203605.7761246427</v>
       </c>
       <c r="K228"/>
@@ -11836,27 +11836,27 @@
       <c r="C229" s="19"/>
       <c r="D229" s="19"/>
       <c r="E229" s="15">
-        <f t="shared" ref="E229:J229" si="76">+E227+E228</f>
+        <f t="shared" ref="E229:J229" si="75">+E227+E228</f>
         <v>189062.5</v>
       </c>
       <c r="F229" s="15">
-        <f t="shared" si="76"/>
+        <f t="shared" si="75"/>
         <v>509996.09375</v>
       </c>
       <c r="G229" s="15">
-        <f t="shared" si="76"/>
+        <f t="shared" si="75"/>
         <v>1007292.38671875</v>
       </c>
       <c r="H229" s="15">
-        <f t="shared" si="76"/>
+        <f t="shared" si="75"/>
         <v>1741376.0285195312</v>
       </c>
       <c r="I229" s="15">
-        <f t="shared" si="76"/>
+        <f t="shared" si="75"/>
         <v>2794483.4956371528</v>
       </c>
       <c r="J229" s="15">
-        <f t="shared" si="76"/>
+        <f t="shared" si="75"/>
         <v>4278743.7219310841</v>
       </c>
       <c r="K229"/>
@@ -12048,23 +12048,23 @@
         <v>37812.5</v>
       </c>
       <c r="F239" s="15">
-        <f t="shared" ref="F239:J239" si="77">SUM(F232:F238)</f>
+        <f t="shared" ref="F239:J239" si="76">SUM(F232:F238)</f>
         <v>109561.71875</v>
       </c>
       <c r="G239" s="15">
-        <f t="shared" si="77"/>
+        <f t="shared" si="76"/>
         <v>230933.32109375001</v>
       </c>
       <c r="H239" s="15">
-        <f t="shared" si="77"/>
+        <f t="shared" si="76"/>
         <v>423936.71367265622</v>
       </c>
       <c r="I239" s="15">
-        <f t="shared" si="77"/>
+        <f t="shared" si="76"/>
         <v>719345.54983071168</v>
       </c>
       <c r="J239" s="15">
-        <f t="shared" si="77"/>
+        <f t="shared" si="76"/>
         <v>1267566.5241225134</v>
       </c>
       <c r="K239"/>
@@ -12088,27 +12088,27 @@
       <c r="C241" s="19"/>
       <c r="D241" s="19"/>
       <c r="E241" s="15">
-        <f t="shared" ref="E241:J241" si="78">E229-E239</f>
+        <f t="shared" ref="E241:J241" si="77">E229-E239</f>
         <v>151250</v>
       </c>
       <c r="F241" s="15">
-        <f t="shared" si="78"/>
+        <f t="shared" si="77"/>
         <v>400434.375</v>
       </c>
       <c r="G241" s="15">
-        <f t="shared" si="78"/>
+        <f t="shared" si="77"/>
         <v>776359.06562500005</v>
       </c>
       <c r="H241" s="15">
-        <f t="shared" si="78"/>
+        <f t="shared" si="77"/>
         <v>1317439.3148468751</v>
       </c>
       <c r="I241" s="15">
-        <f t="shared" si="78"/>
+        <f t="shared" si="77"/>
         <v>2075137.9458064411</v>
       </c>
       <c r="J241" s="15">
-        <f t="shared" si="78"/>
+        <f t="shared" si="77"/>
         <v>3011177.1978085707</v>
       </c>
       <c r="K241"/>
@@ -12155,23 +12155,23 @@
         <v>0</v>
       </c>
       <c r="F245" s="3">
-        <f t="shared" ref="F245:J245" si="79">+E251</f>
+        <f t="shared" ref="F245:J245" si="78">+E251</f>
         <v>0</v>
       </c>
       <c r="G245" s="3">
-        <f t="shared" si="79"/>
+        <f t="shared" si="78"/>
         <v>0</v>
       </c>
       <c r="H245" s="3">
-        <f t="shared" si="79"/>
+        <f t="shared" si="78"/>
         <v>0</v>
       </c>
       <c r="I245" s="3">
-        <f t="shared" si="79"/>
+        <f t="shared" si="78"/>
         <v>0</v>
       </c>
       <c r="J245" s="3">
-        <f t="shared" si="79"/>
+        <f t="shared" si="78"/>
         <v>0</v>
       </c>
       <c r="K245"/>
@@ -12216,27 +12216,27 @@
       <c r="C247" s="19"/>
       <c r="D247" s="19"/>
       <c r="E247" s="15">
-        <f t="shared" ref="E247:J247" si="80">SUM(E245:E246)</f>
+        <f t="shared" ref="E247:J247" si="79">SUM(E245:E246)</f>
         <v>0</v>
       </c>
       <c r="F247" s="15">
-        <f t="shared" si="80"/>
+        <f t="shared" si="79"/>
         <v>0</v>
       </c>
       <c r="G247" s="15">
-        <f t="shared" si="80"/>
+        <f t="shared" si="79"/>
         <v>0</v>
       </c>
       <c r="H247" s="15">
-        <f t="shared" si="80"/>
+        <f t="shared" si="79"/>
         <v>0</v>
       </c>
       <c r="I247" s="15">
-        <f t="shared" si="80"/>
+        <f t="shared" si="79"/>
         <v>0</v>
       </c>
       <c r="J247" s="15">
-        <f t="shared" si="80"/>
+        <f t="shared" si="79"/>
         <v>0</v>
       </c>
       <c r="K247"/>
@@ -12250,27 +12250,27 @@
       </c>
       <c r="B248" s="35"/>
       <c r="E248" s="3">
-        <f t="shared" ref="E248:J248" si="81">IF(E2&lt;$D$120+$D$122,$D$124,0)</f>
+        <f t="shared" ref="E248:J248" si="80">IF(E2&lt;$D$120+$D$122,$D$124,0)</f>
         <v>0</v>
       </c>
       <c r="F248" s="3">
-        <f t="shared" si="81"/>
+        <f t="shared" si="80"/>
         <v>0</v>
       </c>
       <c r="G248" s="3">
-        <f t="shared" si="81"/>
+        <f t="shared" si="80"/>
         <v>0</v>
       </c>
       <c r="H248" s="3">
-        <f t="shared" si="81"/>
+        <f t="shared" si="80"/>
         <v>0</v>
       </c>
       <c r="I248" s="3">
-        <f t="shared" si="81"/>
+        <f t="shared" si="80"/>
         <v>0</v>
       </c>
       <c r="J248" s="3">
-        <f t="shared" si="81"/>
+        <f t="shared" si="80"/>
         <v>0</v>
       </c>
       <c r="K248"/>
@@ -12284,27 +12284,27 @@
       </c>
       <c r="B249" s="31"/>
       <c r="E249" s="3">
-        <f t="shared" ref="E249:J249" si="82">E247*$D$121</f>
+        <f t="shared" ref="E249:J249" si="81">E247*$D$121</f>
         <v>0</v>
       </c>
       <c r="F249" s="3">
-        <f t="shared" si="82"/>
+        <f t="shared" si="81"/>
         <v>0</v>
       </c>
       <c r="G249" s="3">
-        <f t="shared" si="82"/>
+        <f t="shared" si="81"/>
         <v>0</v>
       </c>
       <c r="H249" s="3">
-        <f t="shared" si="82"/>
+        <f t="shared" si="81"/>
         <v>0</v>
       </c>
       <c r="I249" s="3">
-        <f t="shared" si="82"/>
+        <f t="shared" si="81"/>
         <v>0</v>
       </c>
       <c r="J249" s="3">
-        <f t="shared" si="82"/>
+        <f t="shared" si="81"/>
         <v>0</v>
       </c>
       <c r="K249"/>
@@ -12318,27 +12318,27 @@
       </c>
       <c r="B250" s="31"/>
       <c r="E250" s="3">
-        <f t="shared" ref="E250:J250" si="83">E248+E249</f>
+        <f t="shared" ref="E250:J250" si="82">E248+E249</f>
         <v>0</v>
       </c>
       <c r="F250" s="3">
-        <f t="shared" si="83"/>
+        <f t="shared" si="82"/>
         <v>0</v>
       </c>
       <c r="G250" s="3">
-        <f t="shared" si="83"/>
+        <f t="shared" si="82"/>
         <v>0</v>
       </c>
       <c r="H250" s="3">
-        <f t="shared" si="83"/>
+        <f t="shared" si="82"/>
         <v>0</v>
       </c>
       <c r="I250" s="3">
-        <f t="shared" si="83"/>
+        <f t="shared" si="82"/>
         <v>0</v>
       </c>
       <c r="J250" s="3">
-        <f t="shared" si="83"/>
+        <f t="shared" si="82"/>
         <v>0</v>
       </c>
       <c r="K250"/>
@@ -12362,15 +12362,15 @@
         <v>0</v>
       </c>
       <c r="G251" s="15">
-        <f t="shared" ref="G251:I251" si="84">G245+G250</f>
+        <f t="shared" ref="G251:I251" si="83">G245+G250</f>
         <v>0</v>
       </c>
       <c r="H251" s="15">
-        <f t="shared" si="84"/>
+        <f t="shared" si="83"/>
         <v>0</v>
       </c>
       <c r="I251" s="15">
-        <f t="shared" si="84"/>
+        <f t="shared" si="83"/>
         <v>0</v>
       </c>
       <c r="J251" s="15">
@@ -12417,27 +12417,27 @@
         <v>210</v>
       </c>
       <c r="E255" s="3">
-        <f t="shared" ref="E255:J255" si="85">E147/(E34)</f>
+        <f t="shared" ref="E255:J255" si="84">E147/(E34)</f>
         <v>38.333333333333336</v>
       </c>
       <c r="F255" s="3">
-        <f t="shared" si="85"/>
+        <f t="shared" si="84"/>
         <v>40.250000000000007</v>
       </c>
       <c r="G255" s="3">
-        <f t="shared" si="85"/>
+        <f t="shared" si="84"/>
         <v>42.262500000000003</v>
       </c>
       <c r="H255" s="3">
-        <f t="shared" si="85"/>
+        <f t="shared" si="84"/>
         <v>44.375625000000007</v>
       </c>
       <c r="I255" s="3">
-        <f t="shared" si="85"/>
+        <f t="shared" si="84"/>
         <v>46.594406249999999</v>
       </c>
       <c r="J255" s="3">
-        <f t="shared" si="85"/>
+        <f t="shared" si="84"/>
         <v>48.924126562500007</v>
       </c>
       <c r="K255"/>
@@ -12450,27 +12450,27 @@
         <v>204</v>
       </c>
       <c r="E256" s="3">
-        <f t="shared" ref="E256:J256" si="86">(E152+E147)/E41</f>
+        <f t="shared" ref="E256:J256" si="85">(E152+E147)/E41</f>
         <v>47.75</v>
       </c>
       <c r="F256" s="3">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v>55.56</v>
       </c>
       <c r="G256" s="3">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v>64.300575000000009</v>
       </c>
       <c r="H256" s="3">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v>74.076217875000026</v>
       </c>
       <c r="I256" s="3">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v>85.002850999875051</v>
       </c>
       <c r="J256" s="3">
-        <f t="shared" si="86"/>
+        <f t="shared" si="85"/>
         <v>97.209055687543938</v>
       </c>
       <c r="K256"/>
@@ -12483,27 +12483,27 @@
         <v>22</v>
       </c>
       <c r="E257" s="25">
-        <f t="shared" ref="E257:J257" si="87">E255/E256</f>
+        <f t="shared" ref="E257:J257" si="86">E255/E256</f>
         <v>0.80279232111692844</v>
       </c>
       <c r="F257" s="25">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>0.72444204463642914</v>
       </c>
       <c r="G257" s="25">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>0.65726472897015298</v>
       </c>
       <c r="H257" s="25">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>0.59905360010255504</v>
       </c>
       <c r="I257" s="25">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>0.54815109966215714</v>
       </c>
       <c r="J257" s="25">
-        <f t="shared" si="87"/>
+        <f t="shared" si="86"/>
         <v>0.50328774635724594</v>
       </c>
       <c r="K257"/>
@@ -12523,23 +12523,23 @@
         <v>-412547.94520547945</v>
       </c>
       <c r="F258" s="3">
-        <f t="shared" ref="F258:J258" si="88">F205-F209</f>
+        <f t="shared" ref="F258:J258" si="87">F205-F209</f>
         <v>-446370.34235873283</v>
       </c>
       <c r="G258" s="3">
-        <f t="shared" si="88"/>
+        <f t="shared" si="87"/>
         <v>-297747.09373590659</v>
       </c>
       <c r="H258" s="3">
-        <f t="shared" si="88"/>
+        <f t="shared" si="87"/>
         <v>-40976.20377243415</v>
       </c>
       <c r="I258" s="3">
-        <f t="shared" si="88"/>
+        <f t="shared" si="87"/>
         <v>393955.59403268085</v>
       </c>
       <c r="J258" s="3">
-        <f t="shared" si="88"/>
+        <f t="shared" si="87"/>
         <v>1121357.6289967657</v>
       </c>
       <c r="K258"/>

</xml_diff>